<commit_message>
preparing file and folder system
</commit_message>
<xml_diff>
--- a/Compare ESP vs PC/Com_time_esp32_for_all_feats.xlsx
+++ b/Compare ESP vs PC/Com_time_esp32_for_all_feats.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3zn350-my.sharepoint.com/personal/axilpits_ns824g_onmicrosoft_com/Documents/PlatformIO/PlatformIO/Projects/bad-spine-wearable-1/Compare ESP vs PC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="605" documentId="8_{D3B1A18C-87F8-449B-B64F-9EB70B6639B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7D3FF27-1452-4B7D-82D2-F82CA2494A38}"/>
+  <xr:revisionPtr revIDLastSave="754" documentId="8_{D3B1A18C-87F8-449B-B64F-9EB70B6639B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2DDA215-4347-44B4-BAB3-4ED2AB0C8AFB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{925E18B0-4C29-496B-AC79-8E95804F7CE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Φύλλο1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Φύλλο1!$B$50:$BX$50</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -290,9 +287,6 @@
     <t>measurements</t>
   </si>
   <si>
-    <t>percentage difference (%)</t>
-  </si>
-  <si>
     <t>Compare with window assemble time (in milliseconds)</t>
   </si>
   <si>
@@ -305,10 +299,13 @@
     <t>Mean  Total time in milliseconds</t>
   </si>
   <si>
-    <t>Std of percentage difference</t>
+    <t>Mean information loss  (%)</t>
   </si>
   <si>
-    <t>Mean percentage difference (%)</t>
+    <t>information loss  (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Std information loss </t>
   </si>
 </sst>
 </file>
@@ -316,7 +313,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -402,7 +399,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -457,22 +454,22 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="el-GR" sz="1600"/>
+              <a:rPr lang="el-GR" sz="1400" u="none"/>
               <a:t>Μέση Απώλεια</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="el-GR" sz="1600" baseline="0"/>
+              <a:rPr lang="el-GR" sz="1400" u="none" baseline="0"/>
               <a:t> Πληροφορίας ανά χαρατηριστικό από τον Η/Υ στο </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" sz="1600" baseline="0"/>
+              <a:rPr lang="en-US" sz="1400" u="none" baseline="0"/>
               <a:t>ESP32</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="el-GR" sz="1600" baseline="0"/>
+              <a:rPr lang="el-GR" sz="1400" u="none" baseline="0"/>
               <a:t> </a:t>
             </a:r>
-            <a:endParaRPr lang="el-GR" sz="1600"/>
+            <a:endParaRPr lang="el-GR" sz="1400" u="none"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -480,8 +477,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.35657396273741643"/>
-          <c:y val="8.5178875638841564E-3"/>
+          <c:x val="0.20691413573303338"/>
+          <c:y val="8.8921030670177752E-3"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -517,7 +514,7 @@
     <c:view3D>
       <c:rotX val="15"/>
       <c:rotY val="20"/>
-      <c:rAngAx val="0"/>
+      <c:rAngAx val="1"/>
     </c:view3D>
     <c:floor>
       <c:thickness val="0"/>
@@ -562,15 +559,15 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="2.5432996983751417E-2"/>
-          <c:y val="1.8739405271372807E-2"/>
-          <c:w val="0.95327890048226727"/>
-          <c:h val="0.92494029341521666"/>
+          <c:x val="0.12641909047083402"/>
+          <c:y val="8.1985108121781336E-2"/>
+          <c:w val="0.85463195671969572"/>
+          <c:h val="0.73548387794194592"/>
         </c:manualLayout>
       </c:layout>
       <c:bar3DChart>
         <c:barDir val="col"/>
-        <c:grouping val="stacked"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
@@ -581,16 +578,16 @@
               <c:strCache>
                 <c:ptCount val="75"/>
                 <c:pt idx="0">
-                  <c:v>-0.0202</c:v>
+                  <c:v>-0.020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.4524</c:v>
+                  <c:v>-0.452</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-0.1165</c:v>
+                  <c:v>-0.117</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5556</c:v>
+                  <c:v>0.556</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>#ΔΙΑΙΡ/0!</c:v>
@@ -611,109 +608,109 @@
                   <c:v>#ΔΙΑΙΡ/0!</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.0055</c:v>
+                  <c:v>0.006</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-0.0004</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-0.4991</c:v>
+                  <c:v>-0.499</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.3846</c:v>
+                  <c:v>0.385</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.5000</c:v>
+                  <c:v>0.500</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.0004</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.0833</c:v>
+                  <c:v>0.083</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>4.3333</c:v>
+                  <c:v>4.333</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="45">
                   <c:v>#ΔΙΑΙΡ/0!</c:v>
@@ -734,80 +731,88 @@
                   <c:v>#ΔΙΑΙΡ/0!</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-1.7308</c:v>
+                  <c:v>-1.731</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>1.6667</c:v>
+                  <c:v>1.667</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>0.9091</c:v>
+                  <c:v>0.909</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>3.5714</c:v>
+                  <c:v>3.571</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>1.8155</c:v>
+                  <c:v>1.815</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.0641</c:v>
+                  <c:v>0.064</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-0.1786</c:v>
+                  <c:v>-0.179</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-0.1667</c:v>
+                  <c:v>-0.167</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="63">
                   <c:v>#ΔΙΑΙΡ/0!</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>0.1190</c:v>
+                  <c:v>0.119</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-2.3578</c:v>
+                  <c:v>-2.358</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>0.0040</c:v>
+                  <c:v>0.004</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-1.1794</c:v>
+                  <c:v>-1.179</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>0.0034</c:v>
+                  <c:v>0.003</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.0000</c:v>
+                  <c:v>0.000</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
+          <c:spPr>
+            <a:effectLst/>
+            <a:scene3d>
+              <a:camera prst="orthographicFront"/>
+              <a:lightRig rig="threePt" dir="t"/>
+            </a:scene3d>
+            <a:sp3d prstMaterial="matte"/>
+          </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dPt>
             <c:idx val="0"/>
@@ -821,7 +826,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -841,7 +850,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -861,7 +874,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -881,7 +898,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -901,7 +922,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -921,7 +946,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -943,7 +972,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -965,7 +998,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -987,7 +1024,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1009,7 +1050,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1031,7 +1076,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1053,7 +1102,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1076,7 +1129,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1099,7 +1156,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1122,7 +1183,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1145,7 +1210,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1168,7 +1237,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1191,7 +1264,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1213,7 +1290,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1235,7 +1316,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1257,7 +1342,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1279,7 +1368,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1301,7 +1394,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1323,7 +1420,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1346,7 +1447,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1369,7 +1474,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1392,7 +1501,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1415,7 +1528,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1438,7 +1555,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1461,7 +1582,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1483,7 +1608,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1505,7 +1634,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1527,7 +1660,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1549,7 +1686,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1571,7 +1712,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1593,7 +1738,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1616,7 +1765,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1639,7 +1792,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1662,7 +1819,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1685,7 +1846,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1708,7 +1873,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1731,7 +1900,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1753,7 +1926,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1775,7 +1952,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1797,7 +1978,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1819,7 +2004,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1841,7 +2030,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1863,7 +2056,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1886,7 +2083,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1909,7 +2110,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1932,7 +2137,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1955,7 +2164,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1978,7 +2191,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2001,7 +2218,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2021,7 +2242,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2041,7 +2266,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2061,7 +2290,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2081,7 +2314,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2101,7 +2338,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2121,7 +2362,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2143,7 +2388,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2165,7 +2414,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2187,7 +2440,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2209,7 +2466,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2231,7 +2492,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2253,7 +2518,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2276,7 +2545,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2299,7 +2572,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2322,7 +2599,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2345,7 +2626,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2368,7 +2653,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2391,7 +2680,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2413,7 +2706,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2435,7 +2732,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2457,7 +2758,11 @@
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
-              <a:sp3d/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d prstMaterial="matte"/>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2512,8 +2817,8 @@
               <c:idx val="16"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-5.2779732582688269E-2"/>
-                  <c:y val="-7.0982172799098575E-2"/>
+                  <c:x val="-1.6044994375703038E-2"/>
+                  <c:y val="0.15416942322077945"/>
                 </c:manualLayout>
               </c:layout>
               <c:showLegendKey val="0"/>
@@ -2575,8 +2880,8 @@
               <c:idx val="39"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="5.7471264367816091E-2"/>
-                  <c:y val="-7.3821692220329416E-2"/>
+                  <c:x val="6.1552948738550439E-2"/>
+                  <c:y val="0.10327815709578041"/>
                 </c:manualLayout>
               </c:layout>
               <c:showLegendKey val="0"/>
@@ -2638,46 +2943,10 @@
               <c:idx val="53"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="3.1667839549612949E-2"/>
-                  <c:y val="0.12776831345826234"/>
+                  <c:x val="4.1191601049868666E-2"/>
+                  <c:y val="0.17993747486671249"/>
                 </c:manualLayout>
               </c:layout>
-              <c:spPr>
-                <a:solidFill>
-                  <a:sysClr val="window" lastClr="FFFFFF"/>
-                </a:solidFill>
-                <a:ln>
-                  <a:solidFill>
-                    <a:sysClr val="windowText" lastClr="000000">
-                      <a:lumMod val="25000"/>
-                      <a:lumOff val="75000"/>
-                    </a:sysClr>
-                  </a:solidFill>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                  <a:spAutoFit/>
-                </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="dk1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
               <c:showLegendKey val="0"/>
               <c:showVal val="1"/>
               <c:showCatName val="1"/>
@@ -2685,17 +2954,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                    <a:prstGeom prst="wedgeRectCallout">
-                      <a:avLst/>
-                    </a:prstGeom>
-                    <a:noFill/>
-                    <a:ln>
-                      <a:noFill/>
-                    </a:ln>
-                  </c15:spPr>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000006B-1706-4F02-99CC-9D0E0A08EFB9}"/>
                 </c:ext>
@@ -2705,8 +2964,8 @@
               <c:idx val="57"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-6.6854235585083799E-2"/>
-                  <c:y val="-0.18171493469619535"/>
+                  <c:x val="6.7839627189458254E-2"/>
+                  <c:y val="6.6295993239345929E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:showLegendKey val="0"/>
@@ -2747,8 +3006,8 @@
               <c:idx val="65"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-5.3952615528970294E-2"/>
-                  <c:y val="-5.6785917092561047E-2"/>
+                  <c:x val="-7.1639723605977729E-2"/>
+                  <c:y val="6.951878132202173E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:showLegendKey val="0"/>
@@ -3079,7 +3338,7 @@
             <c:numRef>
               <c:f>Φύλλο1!$B$49:$BX$49</c:f>
               <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="75"/>
                 <c:pt idx="0">
                   <c:v>-2.0232660335692911E-2</c:v>
@@ -3366,8 +3625,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="0.38173858193834143"/>
-              <c:y val="0.90451090334321493"/>
+              <c:x val="0.46337125716428301"/>
+              <c:y val="0.93196824449662075"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -3417,7 +3676,7 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -3454,7 +3713,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="90000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3481,39 +3742,16 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="el-GR" sz="1400"/>
-                  <a:t>Ποσοστό</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="el-GR" sz="1400" baseline="0"/>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:effectLst/>
+                  </a:rPr>
                   <a:t> </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="el-GR" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:sysClr val="windowText" lastClr="000000">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:sysClr>
-                    </a:solidFill>
-                  </a:rPr>
-                  <a:t>(%) </a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="el-GR" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
                     <a:effectLst/>
                   </a:rPr>
-                  <a:t>απώλεια</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="el-GR" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                    <a:effectLst/>
-                  </a:rPr>
-                  <a:t> </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="el-GR" sz="1400" baseline="0"/>
-                  <a:t> πληροφορίας χαρακτηριστικών </a:t>
+                  <a:t>Μέση Απώλεια πληροφορίας (%)</a:t>
                 </a:r>
                 <a:endParaRPr lang="el-GR" sz="1400"/>
               </a:p>
@@ -3523,8 +3761,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="4.6409869948522448E-2"/>
-              <c:y val="0.10403448291280457"/>
+              <c:x val="1.647790454764583E-2"/>
+              <c:y val="0.24132171905200483"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -3556,7 +3794,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3615,12 +3853,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -3805,6 +4038,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3820,6 +4058,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3835,6 +4078,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -3850,6 +4098,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -3865,6 +4118,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -3880,6 +4138,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="6"/>
@@ -3897,6 +4160,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="7"/>
@@ -3914,6 +4182,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="8"/>
@@ -3931,6 +4204,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000011-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="9"/>
@@ -3948,6 +4226,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000013-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="10"/>
@@ -3965,6 +4248,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000015-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="11"/>
@@ -3982,6 +4270,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000017-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="12"/>
@@ -4000,6 +4293,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000019-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="13"/>
@@ -4018,6 +4316,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="14"/>
@@ -4036,6 +4339,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="15"/>
@@ -4054,6 +4362,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="16"/>
@@ -4072,6 +4385,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000021-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="17"/>
@@ -4090,6 +4408,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000023-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="18"/>
@@ -4107,6 +4430,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000025-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="19"/>
@@ -4124,6 +4452,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000027-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="20"/>
@@ -4141,6 +4474,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000029-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="21"/>
@@ -4158,6 +4496,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="22"/>
@@ -4175,6 +4518,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="23"/>
@@ -4192,6 +4540,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="24"/>
@@ -4210,6 +4563,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000031-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="25"/>
@@ -4228,6 +4586,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000033-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="26"/>
@@ -4246,6 +4609,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000035-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="27"/>
@@ -4264,6 +4632,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000037-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="28"/>
@@ -4282,6 +4655,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000039-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="29"/>
@@ -4300,6 +4678,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000003B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="30"/>
@@ -4317,6 +4700,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000003D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="31"/>
@@ -4334,6 +4722,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000003F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="32"/>
@@ -4351,6 +4744,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000041-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="33"/>
@@ -4368,6 +4766,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000043-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="34"/>
@@ -4385,6 +4788,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000045-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="35"/>
@@ -4402,6 +4810,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000047-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="36"/>
@@ -4420,6 +4833,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000049-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="37"/>
@@ -4438,6 +4856,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000004B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="38"/>
@@ -4456,6 +4879,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000004D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="39"/>
@@ -4497,6 +4925,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000051-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="41"/>
@@ -4515,6 +4948,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000053-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="42"/>
@@ -4532,6 +4970,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000055-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="43"/>
@@ -4549,6 +4992,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000057-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="44"/>
@@ -4566,6 +5014,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000059-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="45"/>
@@ -4583,6 +5036,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000005B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="46"/>
@@ -4600,6 +5058,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000005D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="47"/>
@@ -4617,6 +5080,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000005F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="48"/>
@@ -4635,6 +5103,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000061-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="49"/>
@@ -4653,6 +5126,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000063-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="50"/>
@@ -4671,6 +5149,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000065-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="51"/>
@@ -4755,6 +5238,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000006D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="55"/>
@@ -4770,6 +5258,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000006F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="56"/>
@@ -4785,6 +5278,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000071-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="57"/>
@@ -4862,6 +5360,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000079-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="61"/>
@@ -4901,6 +5404,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000007D-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="63"/>
@@ -4918,6 +5426,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000007F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="64"/>
@@ -4935,6 +5448,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000081-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="65"/>
@@ -4975,6 +5493,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000085-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="67"/>
@@ -4993,6 +5516,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000087-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="68"/>
@@ -5011,6 +5539,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000089-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="69"/>
@@ -5029,6 +5562,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000008B-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="70"/>
@@ -5070,6 +5608,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000008F-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="72"/>
@@ -5087,6 +5630,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000091-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="73"/>
@@ -5104,6 +5652,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000093-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="74"/>
@@ -5121,6 +5674,11 @@
               <a:effectLst/>
               <a:sp3d/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000095-3C2E-4885-98BF-24B16EFCE616}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:dLbl>
@@ -5627,7 +6185,7 @@
             <c:numRef>
               <c:f>Φύλλο1!$B$50:$BX$50</c:f>
               <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="75"/>
                 <c:pt idx="0">
                   <c:v>7.559458065579866E-2</c:v>
@@ -6033,12 +6591,16 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="el-GR" sz="1400"/>
-                  <a:t>Τυπική</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="el-GR" sz="1400" baseline="0"/>
-                  <a:t> απόκληση ποσοστιαίας απόκλησης  πληροφορίας</a:t>
+                  <a:rPr lang="el-GR" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                    <a:effectLst/>
+                  </a:rPr>
+                  <a:t>Τυπική Απόκληση  Απώλειας πληροφορίας (%)</a:t>
                 </a:r>
                 <a:endParaRPr lang="el-GR" sz="1400"/>
               </a:p>
@@ -6069,11 +6631,11 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="el-GR"/>
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -6132,12 +6694,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -7242,15 +7799,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
+      <xdr:colOff>365760</xdr:colOff>
       <xdr:row>78</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
-      <xdr:row>102</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7280,13 +7837,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>22860</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>411480</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>320040</xdr:colOff>
       <xdr:row>131</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
@@ -12809,7 +13366,7 @@
     </row>
     <row r="25" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B25" s="2">
         <f>B2-B14</f>
@@ -15941,7 +16498,7 @@
     </row>
     <row r="36" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B36" s="2">
         <f>AVERAGE(B25:B34)</f>
@@ -16328,7 +16885,7 @@
     </row>
     <row r="38" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B38" s="2">
         <f>(B25/B2)*100</f>
@@ -19460,7 +20017,7 @@
     </row>
     <row r="49" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B49" s="8">
         <f xml:space="preserve"> AVERAGE(B38:B47)</f>
@@ -19767,7 +20324,7 @@
     </row>
     <row r="50" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B50" s="8">
         <f>_xlfn.STDEV.P(B38:B47)</f>
@@ -23301,7 +23858,7 @@
     </row>
     <row r="73" spans="1:75" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B73" s="3">
         <f>AVERAGE(B62:B71)/1000</f>
@@ -23460,10 +24017,10 @@
     </row>
     <row r="75" spans="1:75" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B75" s="2">
-        <f>$B$73/(10*103)</f>
+        <f>B73/(C76*103)</f>
         <v>5.8519413592233015E-3</v>
       </c>
       <c r="C75" s="2" t="s">
@@ -23630,7 +24187,7 @@
     <row r="77" spans="1:75" x14ac:dyDescent="0.3">
       <c r="A77" s="7"/>
       <c r="B77" s="4">
-        <f>$B$73/(10*103)</f>
+        <f>B75</f>
         <v>5.8519413592233015E-3</v>
       </c>
       <c r="D77" s="2"/>

</xml_diff>